<commit_message>
Preparar cotizador para Streamlit Cloud
</commit_message>
<xml_diff>
--- a/TABLA_PERSONAL_SHOPPER_COMPLETA.xlsx
+++ b/TABLA_PERSONAL_SHOPPER_COMPLETA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\INFORMACION\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f6fe7c058fce39b/MAESTRIA 2 SEMESTRE/TABLA CALCULO SABADO 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFE50C8-6A73-4807-B61E-3FE49BF3FC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{DAFE50C8-6A73-4807-B61E-3FE49BF3FC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A70A06EB-BE9E-4A89-A8C7-F197D56CDE68}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,6 +29,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -704,7 +707,7 @@
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="21.21875" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
     <col min="4" max="4" width="9.109375" customWidth="1"/>
     <col min="5" max="5" width="20.33203125" customWidth="1"/>
     <col min="6" max="6" width="18.6640625" customWidth="1"/>
@@ -1760,7 +1763,7 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="3" t="str">
-        <f t="shared" ref="G36:G67" si="6">IF(E36="","",E36*F36)</f>
+        <f t="shared" ref="G36:G53" si="6">IF(E36="","",E36*F36)</f>
         <v/>
       </c>
       <c r="H36" s="3" t="str">
@@ -2453,7 +2456,7 @@
         <v>29</v>
       </c>
       <c r="B7" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C7" s="3">
         <v>80000</v>
@@ -2464,7 +2467,7 @@
         <v>30</v>
       </c>
       <c r="B8" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C8" s="3">
         <v>80000</v>
@@ -2475,7 +2478,7 @@
         <v>31</v>
       </c>
       <c r="B9" s="4">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="C9" s="3">
         <v>80000</v>
@@ -2486,7 +2489,7 @@
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C10" s="3">
         <v>80000</v>
@@ -2497,7 +2500,7 @@
         <v>33</v>
       </c>
       <c r="B11" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C11" s="3">
         <v>150000</v>
@@ -2508,7 +2511,7 @@
         <v>34</v>
       </c>
       <c r="B12" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C12" s="3">
         <v>80000</v>
@@ -2519,7 +2522,7 @@
         <v>35</v>
       </c>
       <c r="B13" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C13" s="3">
         <v>100000</v>
@@ -2530,7 +2533,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C14" s="3">
         <v>100000</v>
@@ -2541,7 +2544,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C15" s="3">
         <v>120000</v>
@@ -2552,7 +2555,7 @@
         <v>38</v>
       </c>
       <c r="B16" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C16" s="3">
         <v>100000</v>
@@ -2563,7 +2566,7 @@
         <v>39</v>
       </c>
       <c r="B17" s="4">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="C17" s="3">
         <v>150000</v>
@@ -2574,7 +2577,7 @@
         <v>40</v>
       </c>
       <c r="B18" s="4">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="C18" s="3">
         <v>300000</v>
@@ -2585,7 +2588,7 @@
         <v>41</v>
       </c>
       <c r="B19" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C19" s="3">
         <v>500000</v>
@@ -2596,7 +2599,7 @@
         <v>42</v>
       </c>
       <c r="B20" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C20" s="3">
         <v>50000</v>
@@ -2607,7 +2610,7 @@
         <v>43</v>
       </c>
       <c r="B21" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C21" s="3">
         <v>100000</v>
@@ -2618,7 +2621,7 @@
         <v>44</v>
       </c>
       <c r="B22" s="4">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C22" s="3">
         <v>50000</v>
@@ -2629,7 +2632,7 @@
         <v>45</v>
       </c>
       <c r="B23" s="4">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="C23" s="3">
         <v>50000</v>
@@ -2640,7 +2643,7 @@
         <v>46</v>
       </c>
       <c r="B24" s="4">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="C24" s="3">
         <v>80000</v>
@@ -2651,7 +2654,7 @@
         <v>47</v>
       </c>
       <c r="B25" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C25" s="3">
         <v>80000</v>
@@ -2662,7 +2665,7 @@
         <v>48</v>
       </c>
       <c r="B26" s="4">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="C26" s="3">
         <v>100000</v>
@@ -2673,7 +2676,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C27" s="3">
         <v>80000</v>
@@ -2684,7 +2687,7 @@
         <v>50</v>
       </c>
       <c r="B28" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C28" s="3">
         <v>200000</v>
@@ -2695,7 +2698,7 @@
         <v>51</v>
       </c>
       <c r="B29" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C29" s="3">
         <v>200000</v>
@@ -2706,7 +2709,7 @@
         <v>52</v>
       </c>
       <c r="B30" s="4">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="C30" s="3">
         <v>100000</v>
@@ -2717,7 +2720,7 @@
         <v>53</v>
       </c>
       <c r="B31" s="4">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="C31" s="3">
         <v>100000</v>
@@ -2728,7 +2731,7 @@
         <v>54</v>
       </c>
       <c r="B32" s="4">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="C32" s="3">
         <v>80000</v>
@@ -2739,7 +2742,7 @@
         <v>55</v>
       </c>
       <c r="B33" s="4">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="C33" s="3">
         <v>80000</v>
@@ -2750,7 +2753,7 @@
         <v>56</v>
       </c>
       <c r="B34" s="4">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="C34" s="3">
         <v>200000</v>
@@ -2761,7 +2764,7 @@
         <v>57</v>
       </c>
       <c r="B35" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C35" s="3">
         <v>300000</v>
@@ -2772,7 +2775,7 @@
         <v>58</v>
       </c>
       <c r="B36" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C36" s="3">
         <v>200000</v>
@@ -2783,7 +2786,7 @@
         <v>59</v>
       </c>
       <c r="B37" s="4">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="C37" s="3">
         <v>100000</v>
@@ -2794,7 +2797,7 @@
         <v>60</v>
       </c>
       <c r="B38" s="4">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C38" s="3">
         <v>200000</v>
@@ -2805,7 +2808,7 @@
         <v>61</v>
       </c>
       <c r="B39" s="4">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C39" s="3">
         <v>100000</v>

</xml_diff>